<commit_message>
Update default FDK matrix
</commit_message>
<xml_diff>
--- a/public/matrix_file/fdk_matrix.xlsx
+++ b/public/matrix_file/fdk_matrix.xlsx
@@ -1,27 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\dev\Carie Projects\FDK Triangle\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\dev\Carie Projects\FDK Triangle\fdk-triangulator\public\matrix_file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8CB4B17D-0087-4082-B11C-1A4D2FE3743B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E43257C5-5976-498D-A4E9-0DA7C1CBA81E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="25500" windowHeight="14760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1155" windowWidth="26760" windowHeight="15045" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13002" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12786" uniqueCount="442">
   <si>
     <t>ID</t>
   </si>
@@ -41,6 +40,9 @@
     <t>PDF</t>
   </si>
   <si>
+    <t>Text Entries</t>
+  </si>
+  <si>
     <t>Media Summary</t>
   </si>
   <si>
@@ -51,9 +53,6 @@
   </si>
   <si>
     <t>Last Edit Date</t>
-  </si>
-  <si>
-    <t>Muscles, Fascia, Systems</t>
   </si>
   <si>
     <t>'Voluntary' is a delusion`</t>
@@ -401,16 +400,16 @@
     <t>Pelvic Rotation in Walking: Washing Machine (Axis of the Spine)</t>
   </si>
   <si>
-    <t>https://youtube.com/shorts/KnyXwjBg...</t>
+    <t>https://youtube.com/shorts/KnyXwjBg7oU</t>
   </si>
   <si>
-    <t>https://youtube.com/shorts/Vghw7RvR...</t>
+    <t>https://youtube.com/shorts/Vqhw7RvRLvY</t>
   </si>
   <si>
-    <t>https://youtube.com/shorts/n06rQQSk...</t>
+    <t>https://youtube.com/shorts/n06rQQSkuX0</t>
   </si>
   <si>
-    <t>https://youtube.com/shorts/VbpLhius1...</t>
+    <t>https://youtube.com/shorts/VbpLhius1TI</t>
   </si>
   <si>
     <t>https://youtu.be/S8ho624udRc</t>
@@ -1366,14 +1365,14 @@
     <t>6; 8</t>
   </si>
   <si>
-    <t>Entry Text</t>
+    <t>Muscles, Fascia, Systems OH BOY!</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1388,19 +1387,20 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1422,7 +1422,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1729,9 +1729,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:DX118"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="2" max="2" width="51.28515625" customWidth="1"/>
+    <col min="3" max="3" width="50.28515625" customWidth="1"/>
+    <col min="4" max="4" width="34.85546875" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="9" max="9" width="43.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:128" x14ac:dyDescent="0.25">
@@ -1753,20 +1757,20 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>441</v>
+      <c r="G1" t="s">
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L1">
         <v>1</v>
@@ -2125,7 +2129,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>441</v>
       </c>
       <c r="G2" t="s">
         <v>138</v>
@@ -2472,11 +2476,11 @@
       <c r="DT2" t="s">
         <v>273</v>
       </c>
-      <c r="DU2" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV2" t="s">
-        <v>273</v>
+      <c r="DU2">
+        <v>0</v>
+      </c>
+      <c r="DV2">
+        <v>0</v>
       </c>
       <c r="DW2" t="s">
         <v>273</v>
@@ -2837,11 +2841,11 @@
       <c r="DT3" t="s">
         <v>273</v>
       </c>
-      <c r="DU3" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV3" t="s">
-        <v>273</v>
+      <c r="DU3">
+        <v>0</v>
+      </c>
+      <c r="DV3">
+        <v>0</v>
       </c>
       <c r="DW3" t="s">
         <v>273</v>
@@ -3202,11 +3206,11 @@
       <c r="DT4" t="s">
         <v>273</v>
       </c>
-      <c r="DU4" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV4" t="s">
-        <v>273</v>
+      <c r="DU4">
+        <v>0</v>
+      </c>
+      <c r="DV4">
+        <v>0</v>
       </c>
       <c r="DW4" t="s">
         <v>273</v>
@@ -3567,11 +3571,11 @@
       <c r="DT5" t="s">
         <v>273</v>
       </c>
-      <c r="DU5" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV5" t="s">
-        <v>273</v>
+      <c r="DU5">
+        <v>0</v>
+      </c>
+      <c r="DV5">
+        <v>0</v>
       </c>
       <c r="DW5" t="s">
         <v>273</v>
@@ -3932,11 +3936,11 @@
       <c r="DT6" t="s">
         <v>273</v>
       </c>
-      <c r="DU6" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV6" t="s">
-        <v>273</v>
+      <c r="DU6">
+        <v>0</v>
+      </c>
+      <c r="DV6">
+        <v>0</v>
       </c>
       <c r="DW6" t="s">
         <v>273</v>
@@ -4297,11 +4301,11 @@
       <c r="DT7" t="s">
         <v>273</v>
       </c>
-      <c r="DU7" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV7" t="s">
-        <v>273</v>
+      <c r="DU7">
+        <v>0</v>
+      </c>
+      <c r="DV7">
+        <v>0</v>
       </c>
       <c r="DW7" t="s">
         <v>273</v>
@@ -4662,11 +4666,11 @@
       <c r="DT8" t="s">
         <v>273</v>
       </c>
-      <c r="DU8" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV8" t="s">
-        <v>273</v>
+      <c r="DU8">
+        <v>0</v>
+      </c>
+      <c r="DV8">
+        <v>0</v>
       </c>
       <c r="DW8" t="s">
         <v>273</v>
@@ -5027,11 +5031,11 @@
       <c r="DT9" t="s">
         <v>273</v>
       </c>
-      <c r="DU9" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV9" t="s">
-        <v>273</v>
+      <c r="DU9">
+        <v>0</v>
+      </c>
+      <c r="DV9">
+        <v>0</v>
       </c>
       <c r="DW9" t="s">
         <v>273</v>
@@ -5392,11 +5396,11 @@
       <c r="DT10" t="s">
         <v>273</v>
       </c>
-      <c r="DU10" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV10" t="s">
-        <v>273</v>
+      <c r="DU10">
+        <v>0</v>
+      </c>
+      <c r="DV10">
+        <v>0</v>
       </c>
       <c r="DW10" t="s">
         <v>273</v>
@@ -5757,11 +5761,11 @@
       <c r="DT11" t="s">
         <v>273</v>
       </c>
-      <c r="DU11" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV11" t="s">
-        <v>273</v>
+      <c r="DU11">
+        <v>0</v>
+      </c>
+      <c r="DV11">
+        <v>0</v>
       </c>
       <c r="DW11" t="s">
         <v>273</v>
@@ -6122,11 +6126,11 @@
       <c r="DT12" t="s">
         <v>273</v>
       </c>
-      <c r="DU12" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV12" t="s">
-        <v>273</v>
+      <c r="DU12">
+        <v>0</v>
+      </c>
+      <c r="DV12">
+        <v>0</v>
       </c>
       <c r="DW12" t="s">
         <v>273</v>
@@ -6487,11 +6491,11 @@
       <c r="DT13" t="s">
         <v>273</v>
       </c>
-      <c r="DU13" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV13" t="s">
-        <v>273</v>
+      <c r="DU13">
+        <v>0</v>
+      </c>
+      <c r="DV13">
+        <v>0</v>
       </c>
       <c r="DW13" t="s">
         <v>273</v>
@@ -6852,11 +6856,11 @@
       <c r="DT14" t="s">
         <v>273</v>
       </c>
-      <c r="DU14" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV14" t="s">
-        <v>273</v>
+      <c r="DU14">
+        <v>0</v>
+      </c>
+      <c r="DV14">
+        <v>0</v>
       </c>
       <c r="DW14" t="s">
         <v>273</v>
@@ -7217,11 +7221,11 @@
       <c r="DT15" t="s">
         <v>273</v>
       </c>
-      <c r="DU15" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV15" t="s">
-        <v>273</v>
+      <c r="DU15">
+        <v>0</v>
+      </c>
+      <c r="DV15">
+        <v>0</v>
       </c>
       <c r="DW15" t="s">
         <v>273</v>
@@ -7582,11 +7586,11 @@
       <c r="DT16" t="s">
         <v>273</v>
       </c>
-      <c r="DU16" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV16" t="s">
-        <v>273</v>
+      <c r="DU16">
+        <v>0</v>
+      </c>
+      <c r="DV16">
+        <v>0</v>
       </c>
       <c r="DW16" t="s">
         <v>273</v>
@@ -7947,11 +7951,11 @@
       <c r="DT17" t="s">
         <v>273</v>
       </c>
-      <c r="DU17" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV17" t="s">
-        <v>273</v>
+      <c r="DU17">
+        <v>0</v>
+      </c>
+      <c r="DV17">
+        <v>0</v>
       </c>
       <c r="DW17" t="s">
         <v>273</v>
@@ -8312,11 +8316,11 @@
       <c r="DT18" t="s">
         <v>273</v>
       </c>
-      <c r="DU18" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV18" t="s">
-        <v>273</v>
+      <c r="DU18">
+        <v>0</v>
+      </c>
+      <c r="DV18">
+        <v>0</v>
       </c>
       <c r="DW18" t="s">
         <v>273</v>
@@ -8677,11 +8681,11 @@
       <c r="DT19" t="s">
         <v>273</v>
       </c>
-      <c r="DU19" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV19" t="s">
-        <v>273</v>
+      <c r="DU19">
+        <v>0</v>
+      </c>
+      <c r="DV19">
+        <v>0</v>
       </c>
       <c r="DW19" t="s">
         <v>273</v>
@@ -9042,11 +9046,11 @@
       <c r="DT20" t="s">
         <v>273</v>
       </c>
-      <c r="DU20" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV20" t="s">
-        <v>273</v>
+      <c r="DU20">
+        <v>0</v>
+      </c>
+      <c r="DV20">
+        <v>0</v>
       </c>
       <c r="DW20" t="s">
         <v>273</v>
@@ -9407,11 +9411,11 @@
       <c r="DT21" t="s">
         <v>273</v>
       </c>
-      <c r="DU21" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV21" t="s">
-        <v>273</v>
+      <c r="DU21">
+        <v>0</v>
+      </c>
+      <c r="DV21">
+        <v>0</v>
       </c>
       <c r="DW21" t="s">
         <v>273</v>
@@ -9772,11 +9776,11 @@
       <c r="DT22" t="s">
         <v>280</v>
       </c>
-      <c r="DU22" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV22" t="s">
-        <v>273</v>
+      <c r="DU22">
+        <v>0</v>
+      </c>
+      <c r="DV22">
+        <v>0</v>
       </c>
       <c r="DW22" t="s">
         <v>273</v>
@@ -10137,11 +10141,11 @@
       <c r="DT23" t="s">
         <v>273</v>
       </c>
-      <c r="DU23" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV23" t="s">
-        <v>273</v>
+      <c r="DU23">
+        <v>0</v>
+      </c>
+      <c r="DV23">
+        <v>0</v>
       </c>
       <c r="DW23" t="s">
         <v>273</v>
@@ -10502,11 +10506,11 @@
       <c r="DT24" t="s">
         <v>273</v>
       </c>
-      <c r="DU24" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV24" t="s">
-        <v>273</v>
+      <c r="DU24">
+        <v>0</v>
+      </c>
+      <c r="DV24">
+        <v>0</v>
       </c>
       <c r="DW24" t="s">
         <v>273</v>
@@ -10867,11 +10871,11 @@
       <c r="DT25" t="s">
         <v>273</v>
       </c>
-      <c r="DU25" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV25" t="s">
-        <v>273</v>
+      <c r="DU25">
+        <v>0</v>
+      </c>
+      <c r="DV25">
+        <v>0</v>
       </c>
       <c r="DW25" t="s">
         <v>273</v>
@@ -11232,11 +11236,11 @@
       <c r="DT26" t="s">
         <v>273</v>
       </c>
-      <c r="DU26" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV26" t="s">
-        <v>273</v>
+      <c r="DU26">
+        <v>0</v>
+      </c>
+      <c r="DV26">
+        <v>0</v>
       </c>
       <c r="DW26" t="s">
         <v>273</v>
@@ -11597,11 +11601,11 @@
       <c r="DT27" t="s">
         <v>273</v>
       </c>
-      <c r="DU27" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV27" t="s">
-        <v>273</v>
+      <c r="DU27">
+        <v>0</v>
+      </c>
+      <c r="DV27">
+        <v>0</v>
       </c>
       <c r="DW27" t="s">
         <v>273</v>
@@ -11962,11 +11966,11 @@
       <c r="DT28" t="s">
         <v>273</v>
       </c>
-      <c r="DU28" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV28" t="s">
-        <v>273</v>
+      <c r="DU28">
+        <v>0</v>
+      </c>
+      <c r="DV28">
+        <v>0</v>
       </c>
       <c r="DW28" t="s">
         <v>273</v>
@@ -12327,11 +12331,11 @@
       <c r="DT29" t="s">
         <v>273</v>
       </c>
-      <c r="DU29" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV29" t="s">
-        <v>273</v>
+      <c r="DU29">
+        <v>0</v>
+      </c>
+      <c r="DV29">
+        <v>0</v>
       </c>
       <c r="DW29" t="s">
         <v>273</v>
@@ -12692,11 +12696,11 @@
       <c r="DT30" t="s">
         <v>273</v>
       </c>
-      <c r="DU30" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV30" t="s">
-        <v>273</v>
+      <c r="DU30">
+        <v>0</v>
+      </c>
+      <c r="DV30">
+        <v>0</v>
       </c>
       <c r="DW30" t="s">
         <v>273</v>
@@ -13057,11 +13061,11 @@
       <c r="DT31" t="s">
         <v>273</v>
       </c>
-      <c r="DU31" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV31" t="s">
-        <v>273</v>
+      <c r="DU31">
+        <v>0</v>
+      </c>
+      <c r="DV31">
+        <v>0</v>
       </c>
       <c r="DW31" t="s">
         <v>273</v>
@@ -13422,11 +13426,11 @@
       <c r="DT32" t="s">
         <v>273</v>
       </c>
-      <c r="DU32" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV32" t="s">
-        <v>273</v>
+      <c r="DU32">
+        <v>0</v>
+      </c>
+      <c r="DV32">
+        <v>0</v>
       </c>
       <c r="DW32" t="s">
         <v>273</v>
@@ -13790,11 +13794,11 @@
       <c r="DT33" t="s">
         <v>273</v>
       </c>
-      <c r="DU33" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV33" t="s">
-        <v>273</v>
+      <c r="DU33">
+        <v>0</v>
+      </c>
+      <c r="DV33">
+        <v>0</v>
       </c>
       <c r="DW33" t="s">
         <v>273</v>
@@ -14143,11 +14147,11 @@
       <c r="DT34" t="s">
         <v>273</v>
       </c>
-      <c r="DU34" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV34" t="s">
-        <v>273</v>
+      <c r="DU34">
+        <v>0</v>
+      </c>
+      <c r="DV34">
+        <v>0</v>
       </c>
       <c r="DW34" t="s">
         <v>273</v>
@@ -14508,11 +14512,11 @@
       <c r="DT35" t="s">
         <v>273</v>
       </c>
-      <c r="DU35" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV35" t="s">
-        <v>273</v>
+      <c r="DU35">
+        <v>0</v>
+      </c>
+      <c r="DV35">
+        <v>0</v>
       </c>
       <c r="DW35" t="s">
         <v>273</v>
@@ -14876,11 +14880,11 @@
       <c r="DT36" t="s">
         <v>273</v>
       </c>
-      <c r="DU36" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV36" t="s">
-        <v>273</v>
+      <c r="DU36">
+        <v>0</v>
+      </c>
+      <c r="DV36">
+        <v>0</v>
       </c>
       <c r="DW36" t="s">
         <v>273</v>
@@ -15244,11 +15248,11 @@
       <c r="DT37" t="s">
         <v>273</v>
       </c>
-      <c r="DU37" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV37" t="s">
-        <v>273</v>
+      <c r="DU37">
+        <v>0</v>
+      </c>
+      <c r="DV37">
+        <v>0</v>
       </c>
       <c r="DW37" t="s">
         <v>273</v>
@@ -15612,11 +15616,11 @@
       <c r="DT38" t="s">
         <v>273</v>
       </c>
-      <c r="DU38" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV38" t="s">
-        <v>273</v>
+      <c r="DU38">
+        <v>0</v>
+      </c>
+      <c r="DV38">
+        <v>0</v>
       </c>
       <c r="DW38" t="s">
         <v>273</v>
@@ -15980,11 +15984,11 @@
       <c r="DT39" t="s">
         <v>273</v>
       </c>
-      <c r="DU39" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV39" t="s">
-        <v>273</v>
+      <c r="DU39">
+        <v>0</v>
+      </c>
+      <c r="DV39">
+        <v>0</v>
       </c>
       <c r="DW39" t="s">
         <v>273</v>
@@ -16348,11 +16352,11 @@
       <c r="DT40" t="s">
         <v>273</v>
       </c>
-      <c r="DU40" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV40" t="s">
-        <v>273</v>
+      <c r="DU40">
+        <v>0</v>
+      </c>
+      <c r="DV40">
+        <v>0</v>
       </c>
       <c r="DW40" t="s">
         <v>273</v>
@@ -16716,11 +16720,11 @@
       <c r="DT41" t="s">
         <v>273</v>
       </c>
-      <c r="DU41" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV41" t="s">
-        <v>273</v>
+      <c r="DU41">
+        <v>0</v>
+      </c>
+      <c r="DV41">
+        <v>0</v>
       </c>
       <c r="DW41" t="s">
         <v>273</v>
@@ -17084,11 +17088,11 @@
       <c r="DT42" t="s">
         <v>273</v>
       </c>
-      <c r="DU42" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV42" t="s">
-        <v>273</v>
+      <c r="DU42">
+        <v>0</v>
+      </c>
+      <c r="DV42">
+        <v>0</v>
       </c>
       <c r="DW42" t="s">
         <v>273</v>
@@ -17452,11 +17456,11 @@
       <c r="DT43" t="s">
         <v>273</v>
       </c>
-      <c r="DU43" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV43" t="s">
-        <v>273</v>
+      <c r="DU43">
+        <v>0</v>
+      </c>
+      <c r="DV43">
+        <v>0</v>
       </c>
       <c r="DW43" t="s">
         <v>273</v>
@@ -17820,11 +17824,11 @@
       <c r="DT44" t="s">
         <v>273</v>
       </c>
-      <c r="DU44" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV44" t="s">
-        <v>273</v>
+      <c r="DU44">
+        <v>0</v>
+      </c>
+      <c r="DV44">
+        <v>0</v>
       </c>
       <c r="DW44" t="s">
         <v>273</v>
@@ -18188,11 +18192,11 @@
       <c r="DT45" t="s">
         <v>273</v>
       </c>
-      <c r="DU45" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV45" t="s">
-        <v>273</v>
+      <c r="DU45">
+        <v>0</v>
+      </c>
+      <c r="DV45">
+        <v>0</v>
       </c>
       <c r="DW45" t="s">
         <v>273</v>
@@ -18556,11 +18560,11 @@
       <c r="DT46" t="s">
         <v>273</v>
       </c>
-      <c r="DU46" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV46" t="s">
-        <v>273</v>
+      <c r="DU46">
+        <v>0</v>
+      </c>
+      <c r="DV46">
+        <v>0</v>
       </c>
       <c r="DW46" t="s">
         <v>273</v>
@@ -18924,11 +18928,11 @@
       <c r="DT47" t="s">
         <v>273</v>
       </c>
-      <c r="DU47" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV47" t="s">
-        <v>273</v>
+      <c r="DU47">
+        <v>0</v>
+      </c>
+      <c r="DV47">
+        <v>0</v>
       </c>
       <c r="DW47" t="s">
         <v>273</v>
@@ -19292,11 +19296,11 @@
       <c r="DT48" t="s">
         <v>273</v>
       </c>
-      <c r="DU48" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV48" t="s">
-        <v>273</v>
+      <c r="DU48">
+        <v>0</v>
+      </c>
+      <c r="DV48">
+        <v>0</v>
       </c>
       <c r="DW48" t="s">
         <v>273</v>
@@ -19660,11 +19664,11 @@
       <c r="DT49" t="s">
         <v>273</v>
       </c>
-      <c r="DU49" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV49" t="s">
-        <v>273</v>
+      <c r="DU49">
+        <v>0</v>
+      </c>
+      <c r="DV49">
+        <v>0</v>
       </c>
       <c r="DW49" t="s">
         <v>273</v>
@@ -20028,11 +20032,11 @@
       <c r="DT50" t="s">
         <v>273</v>
       </c>
-      <c r="DU50" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV50" t="s">
-        <v>273</v>
+      <c r="DU50">
+        <v>0</v>
+      </c>
+      <c r="DV50">
+        <v>0</v>
       </c>
       <c r="DW50" t="s">
         <v>273</v>
@@ -20396,11 +20400,11 @@
       <c r="DT51" t="s">
         <v>273</v>
       </c>
-      <c r="DU51" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV51" t="s">
-        <v>273</v>
+      <c r="DU51">
+        <v>0</v>
+      </c>
+      <c r="DV51">
+        <v>0</v>
       </c>
       <c r="DW51" t="s">
         <v>273</v>
@@ -20764,11 +20768,11 @@
       <c r="DT52" t="s">
         <v>273</v>
       </c>
-      <c r="DU52" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV52" t="s">
-        <v>273</v>
+      <c r="DU52">
+        <v>0</v>
+      </c>
+      <c r="DV52">
+        <v>0</v>
       </c>
       <c r="DW52" t="s">
         <v>273</v>
@@ -21132,11 +21136,11 @@
       <c r="DT53" t="s">
         <v>273</v>
       </c>
-      <c r="DU53" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV53" t="s">
-        <v>273</v>
+      <c r="DU53">
+        <v>0</v>
+      </c>
+      <c r="DV53">
+        <v>0</v>
       </c>
       <c r="DW53" t="s">
         <v>273</v>
@@ -21500,11 +21504,11 @@
       <c r="DT54" t="s">
         <v>273</v>
       </c>
-      <c r="DU54" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV54" t="s">
-        <v>273</v>
+      <c r="DU54">
+        <v>0</v>
+      </c>
+      <c r="DV54">
+        <v>0</v>
       </c>
       <c r="DW54" t="s">
         <v>273</v>
@@ -21868,11 +21872,11 @@
       <c r="DT55" t="s">
         <v>273</v>
       </c>
-      <c r="DU55" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV55" t="s">
-        <v>273</v>
+      <c r="DU55">
+        <v>0</v>
+      </c>
+      <c r="DV55">
+        <v>0</v>
       </c>
       <c r="DW55" t="s">
         <v>273</v>
@@ -22236,11 +22240,11 @@
       <c r="DT56" t="s">
         <v>273</v>
       </c>
-      <c r="DU56" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV56" t="s">
-        <v>273</v>
+      <c r="DU56">
+        <v>0</v>
+      </c>
+      <c r="DV56">
+        <v>0</v>
       </c>
       <c r="DW56" t="s">
         <v>273</v>
@@ -22604,11 +22608,11 @@
       <c r="DT57" t="s">
         <v>273</v>
       </c>
-      <c r="DU57" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV57" t="s">
-        <v>273</v>
+      <c r="DU57">
+        <v>0</v>
+      </c>
+      <c r="DV57">
+        <v>0</v>
       </c>
       <c r="DW57" t="s">
         <v>273</v>
@@ -22972,11 +22976,11 @@
       <c r="DT58" t="s">
         <v>273</v>
       </c>
-      <c r="DU58" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV58" t="s">
-        <v>273</v>
+      <c r="DU58">
+        <v>0</v>
+      </c>
+      <c r="DV58">
+        <v>0</v>
       </c>
       <c r="DW58" t="s">
         <v>273</v>
@@ -23340,11 +23344,11 @@
       <c r="DT59" t="s">
         <v>273</v>
       </c>
-      <c r="DU59" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV59" t="s">
-        <v>273</v>
+      <c r="DU59">
+        <v>0</v>
+      </c>
+      <c r="DV59">
+        <v>0</v>
       </c>
       <c r="DW59" t="s">
         <v>273</v>
@@ -23708,11 +23712,11 @@
       <c r="DT60" t="s">
         <v>273</v>
       </c>
-      <c r="DU60" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV60" t="s">
-        <v>273</v>
+      <c r="DU60">
+        <v>0</v>
+      </c>
+      <c r="DV60">
+        <v>0</v>
       </c>
       <c r="DW60" t="s">
         <v>273</v>
@@ -24076,11 +24080,11 @@
       <c r="DT61" t="s">
         <v>273</v>
       </c>
-      <c r="DU61" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV61" t="s">
-        <v>273</v>
+      <c r="DU61">
+        <v>0</v>
+      </c>
+      <c r="DV61">
+        <v>0</v>
       </c>
       <c r="DW61" t="s">
         <v>273</v>
@@ -24444,11 +24448,11 @@
       <c r="DT62" t="s">
         <v>273</v>
       </c>
-      <c r="DU62" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV62" t="s">
-        <v>273</v>
+      <c r="DU62">
+        <v>0</v>
+      </c>
+      <c r="DV62">
+        <v>0</v>
       </c>
       <c r="DW62" t="s">
         <v>273</v>
@@ -24812,11 +24816,11 @@
       <c r="DT63" t="s">
         <v>273</v>
       </c>
-      <c r="DU63" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV63" t="s">
-        <v>273</v>
+      <c r="DU63">
+        <v>0</v>
+      </c>
+      <c r="DV63">
+        <v>0</v>
       </c>
       <c r="DW63" t="s">
         <v>273</v>
@@ -25180,11 +25184,11 @@
       <c r="DT64" t="s">
         <v>273</v>
       </c>
-      <c r="DU64" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV64" t="s">
-        <v>273</v>
+      <c r="DU64">
+        <v>0</v>
+      </c>
+      <c r="DV64">
+        <v>0</v>
       </c>
       <c r="DW64" t="s">
         <v>273</v>
@@ -25548,11 +25552,11 @@
       <c r="DT65" t="s">
         <v>273</v>
       </c>
-      <c r="DU65" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV65" t="s">
-        <v>273</v>
+      <c r="DU65">
+        <v>0</v>
+      </c>
+      <c r="DV65">
+        <v>0</v>
       </c>
       <c r="DW65" t="s">
         <v>273</v>
@@ -25916,11 +25920,11 @@
       <c r="DT66" t="s">
         <v>273</v>
       </c>
-      <c r="DU66" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV66" t="s">
-        <v>273</v>
+      <c r="DU66">
+        <v>0</v>
+      </c>
+      <c r="DV66">
+        <v>0</v>
       </c>
       <c r="DW66" t="s">
         <v>273</v>
@@ -26284,11 +26288,11 @@
       <c r="DT67" t="s">
         <v>273</v>
       </c>
-      <c r="DU67" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV67" t="s">
-        <v>273</v>
+      <c r="DU67">
+        <v>0</v>
+      </c>
+      <c r="DV67">
+        <v>0</v>
       </c>
       <c r="DW67" t="s">
         <v>273</v>
@@ -26652,11 +26656,11 @@
       <c r="DT68" t="s">
         <v>273</v>
       </c>
-      <c r="DU68" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV68" t="s">
-        <v>273</v>
+      <c r="DU68">
+        <v>0</v>
+      </c>
+      <c r="DV68">
+        <v>0</v>
       </c>
       <c r="DW68" t="s">
         <v>273</v>
@@ -27020,11 +27024,11 @@
       <c r="DT69" t="s">
         <v>273</v>
       </c>
-      <c r="DU69" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV69" t="s">
-        <v>273</v>
+      <c r="DU69">
+        <v>0</v>
+      </c>
+      <c r="DV69">
+        <v>0</v>
       </c>
       <c r="DW69" t="s">
         <v>273</v>
@@ -27388,11 +27392,11 @@
       <c r="DT70" t="s">
         <v>273</v>
       </c>
-      <c r="DU70" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV70" t="s">
-        <v>273</v>
+      <c r="DU70">
+        <v>0</v>
+      </c>
+      <c r="DV70">
+        <v>0</v>
       </c>
       <c r="DW70" t="s">
         <v>273</v>
@@ -27756,11 +27760,11 @@
       <c r="DT71" t="s">
         <v>273</v>
       </c>
-      <c r="DU71" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV71" t="s">
-        <v>273</v>
+      <c r="DU71">
+        <v>0</v>
+      </c>
+      <c r="DV71">
+        <v>0</v>
       </c>
       <c r="DW71" t="s">
         <v>273</v>
@@ -28124,11 +28128,11 @@
       <c r="DT72" t="s">
         <v>273</v>
       </c>
-      <c r="DU72" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV72" t="s">
-        <v>273</v>
+      <c r="DU72">
+        <v>0</v>
+      </c>
+      <c r="DV72">
+        <v>0</v>
       </c>
       <c r="DW72" t="s">
         <v>273</v>
@@ -28492,11 +28496,11 @@
       <c r="DT73" t="s">
         <v>273</v>
       </c>
-      <c r="DU73" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV73" t="s">
-        <v>273</v>
+      <c r="DU73">
+        <v>0</v>
+      </c>
+      <c r="DV73">
+        <v>0</v>
       </c>
       <c r="DW73" t="s">
         <v>273</v>
@@ -28860,11 +28864,11 @@
       <c r="DT74" t="s">
         <v>273</v>
       </c>
-      <c r="DU74" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV74" t="s">
-        <v>273</v>
+      <c r="DU74">
+        <v>0</v>
+      </c>
+      <c r="DV74">
+        <v>0</v>
       </c>
       <c r="DW74" t="s">
         <v>273</v>
@@ -29228,11 +29232,11 @@
       <c r="DT75" t="s">
         <v>273</v>
       </c>
-      <c r="DU75" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV75" t="s">
-        <v>273</v>
+      <c r="DU75">
+        <v>0</v>
+      </c>
+      <c r="DV75">
+        <v>0</v>
       </c>
       <c r="DW75" t="s">
         <v>273</v>
@@ -29596,11 +29600,11 @@
       <c r="DT76" t="s">
         <v>273</v>
       </c>
-      <c r="DU76" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV76" t="s">
-        <v>273</v>
+      <c r="DU76">
+        <v>0</v>
+      </c>
+      <c r="DV76">
+        <v>0</v>
       </c>
       <c r="DW76" t="s">
         <v>273</v>
@@ -29964,11 +29968,11 @@
       <c r="DT77" t="s">
         <v>273</v>
       </c>
-      <c r="DU77" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV77" t="s">
-        <v>273</v>
+      <c r="DU77">
+        <v>0</v>
+      </c>
+      <c r="DV77">
+        <v>0</v>
       </c>
       <c r="DW77" t="s">
         <v>273</v>
@@ -30332,11 +30336,11 @@
       <c r="DT78" t="s">
         <v>273</v>
       </c>
-      <c r="DU78" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV78" t="s">
-        <v>273</v>
+      <c r="DU78">
+        <v>0</v>
+      </c>
+      <c r="DV78">
+        <v>0</v>
       </c>
       <c r="DW78" t="s">
         <v>273</v>
@@ -30700,11 +30704,11 @@
       <c r="DT79" t="s">
         <v>273</v>
       </c>
-      <c r="DU79" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV79" t="s">
-        <v>273</v>
+      <c r="DU79">
+        <v>0</v>
+      </c>
+      <c r="DV79">
+        <v>0</v>
       </c>
       <c r="DW79" t="s">
         <v>273</v>
@@ -31068,11 +31072,11 @@
       <c r="DT80" t="s">
         <v>273</v>
       </c>
-      <c r="DU80" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV80" t="s">
-        <v>273</v>
+      <c r="DU80">
+        <v>0</v>
+      </c>
+      <c r="DV80">
+        <v>0</v>
       </c>
       <c r="DW80" t="s">
         <v>273</v>
@@ -31436,11 +31440,11 @@
       <c r="DT81" t="s">
         <v>273</v>
       </c>
-      <c r="DU81" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV81" t="s">
-        <v>273</v>
+      <c r="DU81">
+        <v>0</v>
+      </c>
+      <c r="DV81">
+        <v>0</v>
       </c>
       <c r="DW81" t="s">
         <v>273</v>
@@ -31789,11 +31793,11 @@
       <c r="DT82" t="s">
         <v>273</v>
       </c>
-      <c r="DU82" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV82" t="s">
-        <v>273</v>
+      <c r="DU82">
+        <v>0</v>
+      </c>
+      <c r="DV82">
+        <v>0</v>
       </c>
       <c r="DW82" t="s">
         <v>273</v>
@@ -32157,11 +32161,11 @@
       <c r="DT83" t="s">
         <v>273</v>
       </c>
-      <c r="DU83" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV83" t="s">
-        <v>273</v>
+      <c r="DU83">
+        <v>0</v>
+      </c>
+      <c r="DV83">
+        <v>0</v>
       </c>
       <c r="DW83" t="s">
         <v>273</v>
@@ -32510,11 +32514,11 @@
       <c r="DT84" t="s">
         <v>273</v>
       </c>
-      <c r="DU84" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV84" t="s">
-        <v>273</v>
+      <c r="DU84">
+        <v>0</v>
+      </c>
+      <c r="DV84">
+        <v>0</v>
       </c>
       <c r="DW84" t="s">
         <v>273</v>
@@ -32878,11 +32882,11 @@
       <c r="DT85" t="s">
         <v>273</v>
       </c>
-      <c r="DU85" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV85" t="s">
-        <v>273</v>
+      <c r="DU85">
+        <v>0</v>
+      </c>
+      <c r="DV85">
+        <v>0</v>
       </c>
       <c r="DW85" t="s">
         <v>273</v>
@@ -33246,11 +33250,11 @@
       <c r="DT86" t="s">
         <v>273</v>
       </c>
-      <c r="DU86" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV86" t="s">
-        <v>273</v>
+      <c r="DU86">
+        <v>0</v>
+      </c>
+      <c r="DV86">
+        <v>0</v>
       </c>
       <c r="DW86" t="s">
         <v>273</v>
@@ -33614,11 +33618,11 @@
       <c r="DT87" t="s">
         <v>273</v>
       </c>
-      <c r="DU87" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV87" t="s">
-        <v>273</v>
+      <c r="DU87">
+        <v>0</v>
+      </c>
+      <c r="DV87">
+        <v>0</v>
       </c>
       <c r="DW87" t="s">
         <v>273</v>
@@ -33982,11 +33986,11 @@
       <c r="DT88" t="s">
         <v>273</v>
       </c>
-      <c r="DU88" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV88" t="s">
-        <v>273</v>
+      <c r="DU88">
+        <v>0</v>
+      </c>
+      <c r="DV88">
+        <v>0</v>
       </c>
       <c r="DW88" t="s">
         <v>273</v>
@@ -34350,11 +34354,11 @@
       <c r="DT89" t="s">
         <v>273</v>
       </c>
-      <c r="DU89" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV89" t="s">
-        <v>273</v>
+      <c r="DU89">
+        <v>0</v>
+      </c>
+      <c r="DV89">
+        <v>0</v>
       </c>
       <c r="DW89" t="s">
         <v>273</v>
@@ -34718,11 +34722,11 @@
       <c r="DT90" t="s">
         <v>273</v>
       </c>
-      <c r="DU90" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV90" t="s">
-        <v>273</v>
+      <c r="DU90">
+        <v>0</v>
+      </c>
+      <c r="DV90">
+        <v>0</v>
       </c>
       <c r="DW90" t="s">
         <v>273</v>
@@ -35068,11 +35072,11 @@
       <c r="DT91" t="s">
         <v>273</v>
       </c>
-      <c r="DU91" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV91" t="s">
-        <v>273</v>
+      <c r="DU91">
+        <v>0</v>
+      </c>
+      <c r="DV91">
+        <v>0</v>
       </c>
       <c r="DW91" t="s">
         <v>273</v>
@@ -35436,11 +35440,11 @@
       <c r="DT92" t="s">
         <v>273</v>
       </c>
-      <c r="DU92" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV92" t="s">
-        <v>273</v>
+      <c r="DU92">
+        <v>0</v>
+      </c>
+      <c r="DV92">
+        <v>0</v>
       </c>
       <c r="DW92" t="s">
         <v>273</v>
@@ -35804,11 +35808,11 @@
       <c r="DT93" t="s">
         <v>273</v>
       </c>
-      <c r="DU93" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV93" t="s">
-        <v>273</v>
+      <c r="DU93">
+        <v>0</v>
+      </c>
+      <c r="DV93">
+        <v>0</v>
       </c>
       <c r="DW93" t="s">
         <v>273</v>
@@ -36172,11 +36176,11 @@
       <c r="DT94" t="s">
         <v>273</v>
       </c>
-      <c r="DU94" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV94" t="s">
-        <v>273</v>
+      <c r="DU94">
+        <v>0</v>
+      </c>
+      <c r="DV94">
+        <v>0</v>
       </c>
       <c r="DW94" t="s">
         <v>273</v>
@@ -36540,11 +36544,11 @@
       <c r="DT95" t="s">
         <v>273</v>
       </c>
-      <c r="DU95" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV95" t="s">
-        <v>273</v>
+      <c r="DU95">
+        <v>0</v>
+      </c>
+      <c r="DV95">
+        <v>0</v>
       </c>
       <c r="DW95" t="s">
         <v>273</v>
@@ -36908,11 +36912,11 @@
       <c r="DT96" t="s">
         <v>273</v>
       </c>
-      <c r="DU96" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV96" t="s">
-        <v>273</v>
+      <c r="DU96">
+        <v>0</v>
+      </c>
+      <c r="DV96">
+        <v>0</v>
       </c>
       <c r="DW96" t="s">
         <v>273</v>
@@ -37276,11 +37280,11 @@
       <c r="DT97" t="s">
         <v>273</v>
       </c>
-      <c r="DU97" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV97" t="s">
-        <v>273</v>
+      <c r="DU97">
+        <v>0</v>
+      </c>
+      <c r="DV97">
+        <v>0</v>
       </c>
       <c r="DW97" t="s">
         <v>273</v>
@@ -37644,11 +37648,11 @@
       <c r="DT98" t="s">
         <v>273</v>
       </c>
-      <c r="DU98" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV98" t="s">
-        <v>273</v>
+      <c r="DU98">
+        <v>0</v>
+      </c>
+      <c r="DV98">
+        <v>0</v>
       </c>
       <c r="DW98" t="s">
         <v>273</v>
@@ -37994,11 +37998,11 @@
       <c r="DT99" t="s">
         <v>273</v>
       </c>
-      <c r="DU99" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV99" t="s">
-        <v>273</v>
+      <c r="DU99">
+        <v>0</v>
+      </c>
+      <c r="DV99">
+        <v>0</v>
       </c>
       <c r="DW99" t="s">
         <v>273</v>
@@ -38344,11 +38348,11 @@
       <c r="DT100" t="s">
         <v>273</v>
       </c>
-      <c r="DU100" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV100" t="s">
-        <v>273</v>
+      <c r="DU100">
+        <v>0</v>
+      </c>
+      <c r="DV100">
+        <v>0</v>
       </c>
       <c r="DW100" t="s">
         <v>273</v>
@@ -38712,11 +38716,11 @@
       <c r="DT101" t="s">
         <v>273</v>
       </c>
-      <c r="DU101" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV101" t="s">
-        <v>273</v>
+      <c r="DU101">
+        <v>0</v>
+      </c>
+      <c r="DV101">
+        <v>0</v>
       </c>
       <c r="DW101" t="s">
         <v>273</v>
@@ -39065,11 +39069,11 @@
       <c r="DT102" t="s">
         <v>273</v>
       </c>
-      <c r="DU102" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV102" t="s">
-        <v>273</v>
+      <c r="DU102">
+        <v>0</v>
+      </c>
+      <c r="DV102">
+        <v>0</v>
       </c>
       <c r="DW102" t="s">
         <v>273</v>
@@ -39421,11 +39425,11 @@
       <c r="DT103" t="s">
         <v>273</v>
       </c>
-      <c r="DU103" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV103" t="s">
-        <v>273</v>
+      <c r="DU103">
+        <v>0</v>
+      </c>
+      <c r="DV103">
+        <v>0</v>
       </c>
       <c r="DW103" t="s">
         <v>273</v>
@@ -39789,11 +39793,11 @@
       <c r="DT104" t="s">
         <v>273</v>
       </c>
-      <c r="DU104" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV104" t="s">
-        <v>273</v>
+      <c r="DU104">
+        <v>0</v>
+      </c>
+      <c r="DV104">
+        <v>0</v>
       </c>
       <c r="DW104" t="s">
         <v>273</v>
@@ -40157,11 +40161,11 @@
       <c r="DT105" t="s">
         <v>273</v>
       </c>
-      <c r="DU105" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV105" t="s">
-        <v>273</v>
+      <c r="DU105">
+        <v>0</v>
+      </c>
+      <c r="DV105">
+        <v>0</v>
       </c>
       <c r="DW105" t="s">
         <v>273</v>
@@ -40525,11 +40529,11 @@
       <c r="DT106" t="s">
         <v>273</v>
       </c>
-      <c r="DU106" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV106" t="s">
-        <v>273</v>
+      <c r="DU106">
+        <v>0</v>
+      </c>
+      <c r="DV106">
+        <v>0</v>
       </c>
       <c r="DW106" t="s">
         <v>273</v>
@@ -40875,11 +40879,11 @@
       <c r="DT107" t="s">
         <v>273</v>
       </c>
-      <c r="DU107" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV107" t="s">
-        <v>273</v>
+      <c r="DU107">
+        <v>0</v>
+      </c>
+      <c r="DV107">
+        <v>0</v>
       </c>
       <c r="DW107" t="s">
         <v>273</v>
@@ -41243,11 +41247,11 @@
       <c r="DT108" t="s">
         <v>273</v>
       </c>
-      <c r="DU108" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV108" t="s">
-        <v>273</v>
+      <c r="DU108">
+        <v>0</v>
+      </c>
+      <c r="DV108">
+        <v>0</v>
       </c>
       <c r="DW108" t="s">
         <v>273</v>
@@ -41596,11 +41600,11 @@
       <c r="DT109" t="s">
         <v>273</v>
       </c>
-      <c r="DU109" t="s">
-        <v>273</v>
-      </c>
-      <c r="DV109" t="s">
-        <v>273</v>
+      <c r="DU109">
+        <v>0</v>
+      </c>
+      <c r="DV109">
+        <v>0</v>
       </c>
       <c r="DW109" t="s">
         <v>273</v>
@@ -43106,7 +43110,7 @@
       <c r="A114">
         <v>111</v>
       </c>
-      <c r="B114" t="s">
+      <c r="B114" s="2" t="s">
         <v>121</v>
       </c>
       <c r="D114" s="1" t="s">

</xml_diff>

<commit_message>
Render content links from matrix text
</commit_message>
<xml_diff>
--- a/public/matrix_file/fdk_matrix.xlsx
+++ b/public/matrix_file/fdk_matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\dev\Carie Projects\FDK Triangle\fdk-triangulator\public\matrix_file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E08B5AEA-039D-4BAA-B9F4-107C3CA8BB40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE8EBB24-04AE-46D0-9D0C-C3051FD265A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1140" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1366,10 +1366,6 @@
     <t>Navigation System: Very Feldenkraisian</t>
   </si>
   <si>
-    <t>The philosophy for our navigation system is resonant with the Feldenkrais method. It emphasizes exploration. Just as a Feldenkrais lesson Carie ostensibly teaches is actually your lesson, this 'Book of Feldenkrais' is your book. You get choose where you want to meander. In computer terms, this is a berry-picking approach—you create your own path on the hillside as you choose the next juicy idea that you are interested in exploring. For more on 'findability' see Ambient Findability (Morville) — https://www.alibris.com/Ambient-Findability-What-We-Find-Changes-Who-We-Become-Peter-Morville/book/40772935
-Our approach is certainly is non-linear!</t>
-  </si>
-  <si>
     <t>Navigation</t>
   </si>
   <si>
@@ -1594,6 +1590,10 @@
   </si>
   <si>
     <t>https://youtube.com/shorts/LjufMKwxB9A</t>
+  </si>
+  <si>
+    <t>The philosophy for our navigation system is resonant with the Feldenkrais method. It emphasizes exploration. Just as a Feldenkrais lesson Carie ostensibly teaches is actually your lesson, this 'Book of Feldenkrais' is your book. You get choose where you want to meander. In computer terms, this is a berry-picking approach—you create your own path on the hillside as you choose the next juicy idea that you are interested in exploring. For more on [findability](https://www.alibris.com/Ambient-Findability-What-We-Find-Changes-Who-We-Become-Peter-Morville/book/40772935), see Ambient Findability (Morville).
+Our approach is certainly is non-linear!</t>
   </si>
 </sst>
 </file>
@@ -54908,10 +54908,10 @@
         <v>15</v>
       </c>
       <c r="D118" s="8" t="s">
+        <v>515</v>
+      </c>
+      <c r="J118" s="7" t="s">
         <v>444</v>
-      </c>
-      <c r="J118" s="7" t="s">
-        <v>445</v>
       </c>
       <c r="N118" s="9" t="s">
         <v>387</v>
@@ -55325,7 +55325,7 @@
         <v>62</v>
       </c>
       <c r="EU118" s="6" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="EV118" s="6" t="s">
         <v>77</v>
@@ -55357,16 +55357,16 @@
         <v>117</v>
       </c>
       <c r="B119" s="7" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C119" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D119" s="8" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="J119" s="7" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N119" s="9" t="s">
         <v>387</v>
@@ -55806,16 +55806,16 @@
         <v>118</v>
       </c>
       <c r="B120" s="7" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C120" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D120" s="8" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="J120" s="7" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N120" s="9" t="s">
         <v>387</v>
@@ -56270,16 +56270,16 @@
         <v>119</v>
       </c>
       <c r="B121" s="7" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C121" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D121" s="8" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="J121" s="7" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N121" s="9" t="s">
         <v>387</v>
@@ -56719,16 +56719,16 @@
         <v>120</v>
       </c>
       <c r="B122" s="7" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C122" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D122" s="8" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="J122" s="7" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N122" s="9" t="s">
         <v>387</v>
@@ -57168,16 +57168,16 @@
         <v>121</v>
       </c>
       <c r="B123" s="7" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C123" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D123" s="8" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="J123" s="7" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N123" s="9" t="s">
         <v>387</v>
@@ -57617,16 +57617,16 @@
         <v>122</v>
       </c>
       <c r="B124" s="7" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C124" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D124" s="8" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="J124" s="7" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N124" s="9" t="s">
         <v>387</v>
@@ -58066,16 +58066,16 @@
         <v>123</v>
       </c>
       <c r="B125" s="7" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="C125" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D125" s="8" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="J125" s="7" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N125" s="9" t="s">
         <v>18</v>
@@ -58515,13 +58515,13 @@
         <v>124</v>
       </c>
       <c r="B126" s="7" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="C126" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D126" s="8" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="J126" s="7" t="s">
         <v>385</v>
@@ -58964,13 +58964,13 @@
         <v>125</v>
       </c>
       <c r="B127" s="7" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="C127" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D127" s="8" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="J127" s="7" t="s">
         <v>385</v>
@@ -59413,13 +59413,13 @@
         <v>126</v>
       </c>
       <c r="B128" s="7" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="C128" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D128" s="8" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="J128" s="7" t="s">
         <v>385</v>
@@ -59862,13 +59862,13 @@
         <v>127</v>
       </c>
       <c r="B129" s="7" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C129" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D129" s="8" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="J129" s="7" t="s">
         <v>385</v>
@@ -60311,13 +60311,13 @@
         <v>128</v>
       </c>
       <c r="B130" s="7" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C130" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D130" s="8" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="J130" s="7" t="s">
         <v>385</v>
@@ -60760,13 +60760,13 @@
         <v>129</v>
       </c>
       <c r="B131" s="7" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="C131" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D131" s="8" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="J131" s="7" t="s">
         <v>385</v>
@@ -61209,13 +61209,13 @@
         <v>130</v>
       </c>
       <c r="B132" s="7" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="C132" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D132" s="8" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="J132" s="7" t="s">
         <v>385</v>
@@ -61658,13 +61658,13 @@
         <v>131</v>
       </c>
       <c r="B133" s="7" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C133" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D133" s="8" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="J133" s="7" t="s">
         <v>385</v>
@@ -62107,13 +62107,13 @@
         <v>132</v>
       </c>
       <c r="B134" s="7" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="C134" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D134" s="8" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="J134" s="7" t="s">
         <v>385</v>
@@ -62556,13 +62556,13 @@
         <v>133</v>
       </c>
       <c r="B135" s="7" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C135" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D135" s="8" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="J135" s="7" t="s">
         <v>385</v>
@@ -63011,13 +63011,13 @@
         <v>134</v>
       </c>
       <c r="B136" s="7" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C136" s="7" t="s">
         <v>15</v>
       </c>
       <c r="D136" s="8" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="J136" s="7" t="s">
         <v>385</v>
@@ -63466,16 +63466,16 @@
         <v>135</v>
       </c>
       <c r="B137" s="6" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="C137" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D137" s="6" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="J137" s="6" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N137" s="6" t="s">
         <v>387</v>
@@ -63901,7 +63901,7 @@
         <v>0</v>
       </c>
       <c r="EY137" s="6" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="EZ137" s="6">
         <v>0</v>
@@ -63921,16 +63921,16 @@
         <v>136</v>
       </c>
       <c r="B138" s="6" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C138" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D138" s="6" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="J138" s="6" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N138" s="6" t="s">
         <v>387</v>
@@ -64284,7 +64284,7 @@
         <v>0</v>
       </c>
       <c r="EA138" s="6" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="EB138" s="6" t="s">
         <v>277</v>
@@ -64370,16 +64370,16 @@
         <v>137</v>
       </c>
       <c r="B139" s="6" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C139" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D139" s="6" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="J139" s="6" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N139" s="6" t="s">
         <v>387</v>
@@ -64819,16 +64819,16 @@
         <v>138</v>
       </c>
       <c r="B140" s="6" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C140" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D140" s="6" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="J140" s="6" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N140" s="6" t="s">
         <v>387</v>
@@ -65268,16 +65268,16 @@
         <v>139</v>
       </c>
       <c r="B141" s="6" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C141" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D141" s="6" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="J141" s="6" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N141" s="6" t="s">
         <v>387</v>
@@ -65717,16 +65717,16 @@
         <v>140</v>
       </c>
       <c r="B142" s="6" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="C142" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D142" s="6" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="J142" s="6" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N142" s="6" t="s">
         <v>387</v>
@@ -66137,7 +66137,7 @@
         <v>0</v>
       </c>
       <c r="ET142" s="6" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="EU142" s="6" t="s">
         <v>71</v>
@@ -66166,16 +66166,16 @@
         <v>141</v>
       </c>
       <c r="B143" s="6" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="C143" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D143" s="6" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="J143" s="6" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N143" s="6" t="s">
         <v>387</v>
@@ -66615,16 +66615,16 @@
         <v>142</v>
       </c>
       <c r="B144" s="6" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="C144" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D144" s="6" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="J144" s="6" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="N144" s="6" t="s">
         <v>387</v>
@@ -67064,19 +67064,19 @@
         <v>147</v>
       </c>
       <c r="B145" s="6" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="C145" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D145" s="6" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="J145" s="6" t="s">
         <v>220</v>
       </c>
       <c r="K145" s="6" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="N145" s="6" t="s">
         <v>387</v>
@@ -67525,19 +67525,19 @@
         <v>148</v>
       </c>
       <c r="B146" s="6" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="C146" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D146" s="6" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="J146" s="6" t="s">
         <v>220</v>
       </c>
       <c r="K146" s="6" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="N146" s="6" t="s">
         <v>387</v>
@@ -67998,19 +67998,19 @@
         <v>149</v>
       </c>
       <c r="B147" s="6" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C147" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D147" s="6" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="J147" s="6" t="s">
         <v>220</v>
       </c>
       <c r="K147" s="6" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="N147" s="6" t="s">
         <v>387</v>
@@ -68465,19 +68465,19 @@
         <v>150</v>
       </c>
       <c r="B148" s="6" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="C148" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D148" s="6" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="J148" s="6" t="s">
         <v>220</v>
       </c>
       <c r="K148" s="6" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="N148" s="6" t="s">
         <v>387</v>
@@ -68932,19 +68932,19 @@
         <v>151</v>
       </c>
       <c r="B149" s="6" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="C149" s="6" t="s">
         <v>15</v>
       </c>
       <c r="D149" s="6" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="J149" s="6" t="s">
         <v>220</v>
       </c>
       <c r="K149" s="6" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="N149" s="6" t="s">
         <v>387</v>
@@ -69408,13 +69408,13 @@
         <v>152</v>
       </c>
       <c r="B150" s="6" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="C150" s="6" t="s">
         <v>400</v>
       </c>
       <c r="F150" s="6" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="J150" s="6" t="s">
         <v>403</v>
@@ -69881,13 +69881,13 @@
         <v>153</v>
       </c>
       <c r="B151" s="6" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="C151" s="6" t="s">
         <v>400</v>
       </c>
       <c r="F151" s="6" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="J151" s="6" t="s">
         <v>403</v>
@@ -70354,13 +70354,13 @@
         <v>154</v>
       </c>
       <c r="B152" s="6" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="C152" s="6" t="s">
         <v>400</v>
       </c>
       <c r="F152" s="6" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="J152" s="6" t="s">
         <v>403</v>

</xml_diff>

<commit_message>
Fix matrix content link syntax
</commit_message>
<xml_diff>
--- a/public/matrix_file/fdk_matrix.xlsx
+++ b/public/matrix_file/fdk_matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\dev\Carie Projects\FDK Triangle\fdk-triangulator\public\matrix_file\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE8EBB24-04AE-46D0-9D0C-C3051FD265A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{908B7313-FDAB-4A29-A9EC-E7C850C5D83C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1140" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1592,7 +1592,7 @@
     <t>https://youtube.com/shorts/LjufMKwxB9A</t>
   </si>
   <si>
-    <t>The philosophy for our navigation system is resonant with the Feldenkrais method. It emphasizes exploration. Just as a Feldenkrais lesson Carie ostensibly teaches is actually your lesson, this 'Book of Feldenkrais' is your book. You get choose where you want to meander. In computer terms, this is a berry-picking approach—you create your own path on the hillside as you choose the next juicy idea that you are interested in exploring. For more on [findability](https://www.alibris.com/Ambient-Findability-What-We-Find-Changes-Who-We-Become-Peter-Morville/book/40772935), see Ambient Findability (Morville).
+    <t>The philosophy for our navigation system is resonant with the Feldenkrais method. It emphasizes exploration. Just as a Feldenkrais lesson Carie ostensibly teaches is actually your lesson, this 'Book of Feldenkrais' is your book. You get choose where you want to meander. In computer terms, this is a berry-picking approach—you create your own path on the hillside as you choose the next juicy idea that you are interested in exploring. For more on findability, see [Ambient Findability(Morville)](https://www.alibris.com/Ambient-Findability-What-We-Find-Changes-Who-We-Become-Peter-Morville/book/40772935).
 Our approach is certainly is non-linear!</t>
   </si>
 </sst>

</xml_diff>